<commit_message>
feat(F-NAR-009): ENE.001-09 et PAR.001
Ouvertures du monde, texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-09.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-09.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Amélie joue avec l'énergie de Loïc</t>
+          <t>Le ballon jaune de la cour</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DIF.BES.001</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +835,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Un ballon jaune attend près du portail. Raphaël joue avec Aniss, qui a beaucoup d'énergie. Ils tapent le ballon à tour de rôle. Raphaël demande à maman quand ça va trop vite.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Amélie est dans la cour. Loïc saute beaucoup. Loïc a de l'énergie. Maman est près du portail. Ce n'est pas une faute. Beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. Amélie joue avec Loïc. Loïc attend son tour. Ils tapent le ballon. Le ballon est doux. On joue ou on attend. On peut demander à un adulte. Maman sourit.</t>
+          <t>Le portail de bois craque un peu. Une feuille jaune tourne dans l'air. Elle tombe sur l'herbe. L'herbe sent la terre mouillée. Un oiseau picore près de la haie. Papa balaie près des caisses. Le balai fait un petit chut-chut. Maman plie un pull sur le banc. Le pull est bleu et doux. Le banc est encore un peu froid. Tu as vu la feuille, Raphaël ? Elle tourne, papa. Elle est toute jaune. En ce moment, Raphaël tient un ballon. Le ballon est jaune aussi. Il est doux sous les doigts. Il sent un peu le soleil. Aniss arrive dans la cour. Aniss saute sur place. Ses chaussures tapent le sol. Ça fait tap, tap, tap. Aniss a de l'énergie. Beaucoup d'énergie. Raphaël le regarde. Tu as vu Aniss ? Il a de l'énergie. Ce n'est pas une faute. Beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. On joue ou on attend. Raphaël pose le ballon un instant. Il attend un petit moment. Aniss saute encore. Puis Aniss s'arrête. Il souffle. Raphaël tend le ballon. Aniss le prend. Ils tapent le ballon. Le ballon fait poum. Poum, poum, sur l'herbe. Bravo, Raphaël. Tu as su attendre. C'est du bon travail. Aniss attend son tour aussi ? Oui, papa. Aniss pose le ballon. Il attend son tour. Raphaël tape le ballon. Le ballon roule vers le banc. Aniss le rattrape. Ils jouent. Plus tard, Aniss saute encore. L'énergie est encore là. Ce n'est pas une faute. Raphaël va vers maman. Il demande à un adulte. Maman, Aniss a de l'énergie. On peut jouer ou attendre. Tu veux un tour plus calme ? On peut s'asseoir un moment. Oui. Ils s'assoient sur le banc. Le bois est lisse. Aniss souffle. Le ballon reste près des pieds. Puis ils reprennent le ballon. À tour de rôle. Bravo, vous deux. Vous avez joué. Vous avez attendu.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,13 +1329,85 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Amélie est dans la cour. Loïc saute beaucoup. Loïc a de l'énergie. Maman est près du portail.
-maman|Ce n'est pas une faute. Beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre.
-narrateur|Amélie joue avec Loïc. Loïc attend son tour. Ils tapent le ballon. Le ballon est doux.
-enfant-f|On joue ou on attend. On peut demander à un adulte. Maman sourit.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|Le portail de bois craque un peu.
+narrateur|Une feuille jaune tourne dans l'air.
+narrateur|Elle tombe sur l'herbe.
+narrateur|L'herbe sent la terre mouillée.
+narrateur|Un oiseau picore près de la haie.
+narrateur|Papa balaie près des caisses.
+narrateur|Le balai fait un petit chut-chut.
+narrateur|Maman plie un pull sur le banc.
+narrateur|Le pull est bleu et doux.
+narrateur|Le banc est encore un peu froid.
+papa|Tu as vu la feuille, Raphaël ?
+enfant-m|Elle tourne, papa.
+maman|Elle est toute jaune.
+narrateur|En ce moment, Raphaël tient un ballon.
+narrateur|Le ballon est jaune aussi.
+narrateur|Il est doux sous les doigts.
+narrateur|Il sent un peu le soleil.
+narrateur|Aniss arrive dans la cour.
+narrateur|Aniss saute sur place.
+narrateur|Ses chaussures tapent le sol.
+narrateur|Ça fait tap, tap, tap.
+narrateur|Aniss a de l'énergie.
+narrateur|Beaucoup d'énergie.
+narrateur|Raphaël le regarde.
+papa|Tu as vu Aniss ?
+papa|Il a de l'énergie.
+maman|Ce n'est pas une faute.
+maman|Beaucoup d'énergie, ce n'est pas une faute.
+maman|On peut jouer.
+maman|On peut attendre.
+papa|On peut demander à un adulte.
+enfant-m|On joue ou on attend.
+narrateur|Raphaël pose le ballon un instant.
+narrateur|Il attend un petit moment.
+narrateur|Aniss saute encore.
+narrateur|Puis Aniss s'arrête.
+narrateur|Il souffle.
+narrateur|Raphaël tend le ballon.
+narrateur|Aniss le prend.
+narrateur|Ils tapent le ballon.
+narrateur|Le ballon fait poum.
+narrateur|Poum, poum, sur l'herbe.
+maman|Bravo, Raphaël.
+maman|Tu as su attendre.
+papa|C'est du bon travail.
+papa|Aniss attend son tour aussi ?
+enfant-m|Oui, papa.
+narrateur|Aniss pose le ballon.
+narrateur|Il attend son tour.
+narrateur|Raphaël tape le ballon.
+narrateur|Le ballon roule vers le banc.
+narrateur|Aniss le rattrape.
+narrateur|Ils jouent.
+narrateur|Plus tard, Aniss saute encore.
+narrateur|L'énergie est encore là.
+narrateur|Ce n'est pas une faute.
+narrateur|Raphaël va vers maman.
+narrateur|Il demande à un adulte.
+enfant-m|Maman, Aniss a de l'énergie.
+maman|On peut jouer ou attendre.
+maman|Tu veux un tour plus calme ?
+papa|On peut s'asseoir un moment.
+enfant-m|Oui.
+narrateur|Ils s'assoient sur le banc.
+narrateur|Le bois est lisse.
+narrateur|Aniss souffle.
+narrateur|Le ballon reste près des pieds.
+narrateur|Puis ils reprennent le ballon.
+narrateur|À tour de rôle.
+maman|Bravo, vous deux.
+papa|Vous avez joué.
+papa|Vous avez attendu.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1343,7 +1432,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Loïc a de l'énergie. Que peut faire Amélie ?</t>
+          <t>Aniss a de l'énergie. Que peut faire Raphaël ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1503,7 +1592,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Loïc a de l'énergie. Que peut faire Amélie ?</t>
+          <t>narrateur|Aniss a de l'énergie.
+narrateur|Que peut faire Raphaël ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1531,7 +1621,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Loïc a de l'énergie. Ce n'est pas une faute. Amélie a joué. Elle a su attendre.</t>
+          <t>Raphaël a joué. Il a su attendre. Il a demandé à un adulte. Aniss a de l'énergie. Ce n'est pas une faute. Bravo, Raphaël. Tu as fait du bon travail. On peut jouer ou attendre. Tu as pensé à Aniss ? Oui. On a attendu notre tour.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1675,7 +1765,17 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Loïc a de l'énergie. Ce n'est pas une faute. Amélie a joué. Elle a su attendre.</t>
+          <t>narrateur|Raphaël a joué.
+narrateur|Il a su attendre.
+narrateur|Il a demandé à un adulte.
+narrateur|Aniss a de l'énergie.
+narrateur|Ce n'est pas une faute.
+maman|Bravo, Raphaël.
+maman|Tu as fait du bon travail.
+papa|On peut jouer ou attendre.
+papa|Tu as pensé à Aniss ?
+enfant-m|Oui.
+enfant-m|On a attendu notre tour.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1703,7 +1803,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la main d'Amélie. Loïc range le ballon.</t>
+          <t>Le soleil baisse un peu. L'herbe est plus fraîche. Maman range le pull bleu. Papa prend la main de Raphaël. Aniss pose le ballon près du portail. Le ballon reste ici ? Il attend demain. Bravo. Vous avez bien joué. Le portail craque encore. Ils rentrent.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1843,7 +1943,17 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman prend la main d'Amélie. Loïc range le ballon.</t>
+          <t>narrateur|Le soleil baisse un peu.
+narrateur|L'herbe est plus fraîche.
+narrateur|Maman range le pull bleu.
+narrateur|Papa prend la main de Raphaël.
+narrateur|Aniss pose le ballon près du portail.
+maman|Le ballon reste ici ?
+enfant-m|Il attend demain.
+papa|Bravo.
+papa|Vous avez bien joué.
+narrateur|Le portail craque encore.
+narrateur|Ils rentrent.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1871,7 +1981,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>On a tapé le ballon. On a attendu. Bravo. Tu as fait du bon travail. L'énergie, ce n'est pas une faute. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2011,7 +2121,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|On a tapé le ballon.
+enfant-m|On a attendu.
+maman|Bravo.
+maman|Tu as fait du bon travail.
+papa|L'énergie, ce n'est pas une faute.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2033,7 +2148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2071,6 +2186,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-09 Le ballon jaune de la cour
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-09.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-09.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'escargot de raisins</t>
+          <t>Le ballon jaune de la cour</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, bol de raisins, four</t>
+          <t>cour, portail de bois, gond, lattes, poussière chaude, mouche, caisse, ballon jaune</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, Amir, papa, maman</t>
+          <t>Raphaël, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut un escargot de raisins sur le gâteau. Amir a de l'énergie. Les raisins roulent. Ils posent un raisin chacun. Le gâteau part au four.</t>
+          <t>Le bois du portail sent le soleil. Sur le gond, un éclat de gond luit. Raphaël veut le ballon jaune, maintenant. Aniss court trop. Le ballon tape le bois. Sourire parti. Papa s'accroupit. Il refuse de foncer. Merci vécu. Le ballon roule sous le portail. Il s'arrête. Un éclat de gond tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La farine a fait un nuage blanc. Le bol de raisins sent le soleil. Un grain colle au bord du bol. La cuillère en bois est encore farinée. Tu as vu le nuage, Victorina ? Il est blanc, papa. Ça sent déjà le gâteau. Je veux un escargot. Un escargot de raisins. Sur le gâteau rond ? Oui. Tout en rond. Papa tapote la pâte. Toc, toc, sur le bois. La pâte est molle et tiède. Elle sent un peu le lait. Maman beurre le moule. Le beurre brille un peu. Le moule est rond et froid. En ce moment, Victorina prend un raisin. Il est lisse et un peu collant. Le premier, au milieu. Comme une tête d'escargot. Elle pose le raisin. Le gâteau est encore pâle. Amir arrive dans la cuisine. Il saute sur place. Ses chaussettes tapent le carrelage. Ça fait tap, tap, tap. Le bol tremble. Des raisins roulent sur la table. Ils partent, papa ! Amir a de l'énergie. Beaucoup d'énergie. Ce n'est pas une faute. Victorina attrape un raisin. Amir saute encore. Le bol glisse un peu.</t>
+          <t>Le bois du portail sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Une latte claque un peu. Le portail est presque fermé. Il claque, maman. Papa tapote le gond. Toc, toc, sur le fer. Tu entends le gond, Raphaël ? Oui, il grince. Maman pose la main sur le bois. Le bois est chaud, un peu rêche. Sur le gond, un éclat de gond luit. Il brille, maman. Tu le vois, sur le gond ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les lattes. La poussière dore, près du mur. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Raphaël ? Un peu. Une mouche visite une chaussure. Elle fait un petit bzz. Elle part. La mouche a fini. Le ballon jaune dort près du mur. En ce moment, Raphaël le prend. Je veux le ballon, maintenant ! Tout de suite ? Oui, papa. Le caoutchouc est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Aniss arrive dans la cour. Il court trop. Il saute près du portail. Le ballon ! Tu viens, Aniss ? Oui. Raphaël pousse le ballon trop vite. Aniss court dessus. Le ballon tape le bois. Il ne roule plus. Oh. Il est tombé. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de gond tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La farine a fait un nuage blanc. Le bol de raisins sent le soleil. Un grain colle au bord du bol. La cuillère en bois est encore farinée. Tu as vu le nuage, Victorina ? Il est blanc, papa. Ça sent déjà le gâteau. Je veux un escargot. Un escargot de raisins. Sur le gâteau rond ? Oui. Tout en rond. Papa tapote la pâte. Toc, toc, sur le bois. La pâte est molle et tiède. Elle sent un peu le lait. Maman beurre le moule. Le beurre brille un peu. Le moule est rond et froid. En ce moment, Victorina prend un raisin. Il est lisse et un peu collant. Le premier, au milieu. Comme une tête d'escargot. Elle pose le raisin. Le gâteau est encore pâle. Amir arrive dans la cuisine. Il saute sur place. Ses chaussettes tapent le carrelage. Ça fait tap, tap, tap. Le bol tremble. Des raisins roulent sur la table. Ils partent, papa ! Amir a de l'énergie. Beaucoup d'énergie. Ce n'est pas une faute. Victorina attrape un raisin. Amir saute encore. Le bol glisse un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois du portail sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Une latte claque un peu. Le portail est presque fermé. Il claque, maman. Papa tapote le gond. Toc, toc, sur le fer. Tu entends le gond, Raphaël ? Oui, il grince. Maman pose la main sur le bois. Le bois est chaud, un peu rêche. Sur le gond, un &lt;emphasis level="moderate"&gt;éclat de gond&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le gond ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les lattes. La poussière dore, près du mur. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Raphaël ? Un peu. Une mouche visite une chaussure. Elle fait un petit bzz. Elle part. La mouche a fini. Le ballon jaune dort près du mur. En ce moment, Raphaël le prend. Je veux le ballon, maintenant ! Tout de suite ? Oui, papa. Le caoutchouc est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Aniss arrive dans la cour. Il court trop. Il saute près du portail. Le ballon ! Tu viens, Aniss ? Oui. Raphaël pousse le ballon trop vite. Aniss court dessus. Le ballon tape le bois. Il ne roule plus. Oh. Il est tombé. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de gond tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Amélie est dans la cour. Loïc saute beaucoup. Loïc a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Maman est près du portail. Maman dit : ce n'est pas une faute. Beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. Amélie joue avec Loïc. Loïc attend son tour. Ils tapent le ballon. Le ballon est doux. Amélie dit : on joue ou on attend. On peut demander à un adulte. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>Le bois du portail sent le soleil. Ça sent le bois, papa. Tu le sens, le bois chaud ? Oui, papa. Une latte claque un peu. Le portail est presque fermé. Il claque, maman. Papa tapote le gond. Toc, toc, sur le fer. Tu entends le gond, Raphaël ? Oui, il grince. Maman pose la main sur le bois. Le bois est chaud, un peu rêche. Sur le gond, un &lt;emphasis&gt;éclat de gond&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le gond ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les lattes. La poussière dore, près du mur. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Raphaël ? Un peu. Une mouche visite une chaussure. Elle fait un petit bzz. Elle part. La mouche a fini. Le ballon jaune dort près du mur. En ce moment, Raphaël le prend. Je veux le ballon, maintenant ! Tout de suite ? Oui, papa. Le caoutchouc est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Aniss arrive dans la cour. Il court trop. Il saute près du portail. Le ballon ! Tu viens, Aniss ? Oui. Raphaël pousse le ballon trop vite. Aniss court dessus. Le ballon tape le bois. Il ne roule plus. Oh. Il est tombé. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de gond tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de gond</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,49 +1324,73 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_ballon_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La farine a fait un nuage blanc.
-narrateur|Le bol de raisins sent le soleil.
-narrateur|Un grain colle au bord du bol.
-narrateur|La cuillère en bois est encore farinée.
-papa|Tu as vu le nuage, Victorina ?
-enfant-f|Il est blanc, papa.
-maman|Ça sent déjà le gâteau.
-enfant-f|Je veux un escargot.
-enfant-f|Un escargot de raisins.
-maman|Sur le gâteau rond ?
-enfant-f|Oui.
-enfant-f|Tout en rond.
-narrateur|Papa tapote la pâte.
-narrateur|Toc, toc, sur le bois.
-narrateur|La pâte est molle et tiède.
-narrateur|Elle sent un peu le lait.
-narrateur|Maman beurre le moule.
-narrateur|Le beurre brille un peu.
-narrateur|Le moule est rond et froid.
-narrateur|En ce moment, Victorina prend un raisin.
-narrateur|Il est lisse et un peu collant.
-enfant-f|Le premier, au milieu.
-papa|Comme une tête d'escargot.
-narrateur|Elle pose le raisin.
-narrateur|Le gâteau est encore pâle.
-narrateur|Amir arrive dans la cuisine.
-narrateur|Il saute sur place.
-narrateur|Ses chaussettes tapent le carrelage.
-narrateur|Ça fait tap, tap, tap.
-narrateur|Le bol tremble.
-narrateur|Des raisins roulent sur la table.
-enfant-f|Ils partent, papa !
-papa|Amir a de l'énergie.
-maman|Beaucoup d'énergie.
-maman|Ce n'est pas une faute.
-narrateur|Victorina attrape un raisin.
-narrateur|Amir saute encore.
-narrateur|Le bol glisse un peu.</t>
+          <t>narrateur|Le bois du portail sent le soleil.
+enfant-m|Ça sent le bois, papa.
+papa|Tu le sens, le bois chaud ?
+enfant-m|Oui, papa.
+narrateur|Une latte claque un peu.
+maman|Le portail est presque fermé.
+enfant-m|Il claque, maman.
+narrateur|Papa tapote le gond.
+narrateur|Toc, toc, sur le fer.
+papa|Tu entends le gond, Raphaël ?
+enfant-m|Oui, il grince.
+narrateur|Maman pose la main sur le bois.
+narrateur|Le bois est chaud, un peu rêche.
+narrateur|Sur le gond, un éclat de gond luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le gond ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse entre les lattes.
+narrateur|La poussière dore, près du mur.
+narrateur|Elle chatouille le pantalon.
+enfant-m|Elle est chaude.
+maman|Tu t'assois, Raphaël ?
+enfant-m|Un peu.
+narrateur|Une mouche visite une chaussure.
+narrateur|Elle fait un petit bzz.
+enfant-m|Elle part.
+papa|La mouche a fini.
+narrateur|Le ballon jaune dort près du mur.
+narrateur|En ce moment, Raphaël le prend.
+enfant-m|Je veux le ballon, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Le caoutchouc est tiède, un peu poudreux.
+maman|Tu le fais rouler ?
+enfant-m|Oui, maman.
+narrateur|Aniss arrive dans la cour.
+narrateur|Il court trop.
+narrateur|Il saute près du portail.
+copain|Le ballon !
+enfant-m|Tu viens, Aniss ?
+copain|Oui.
+narrateur|Raphaël pousse le ballon trop vite.
+narrateur|Aniss court dessus.
+narrateur|Le ballon tape le bois.
+narrateur|Il ne roule plus.
+enfant-m|Oh.
+copain|Il est tombé.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Raphaël ?
+enfant-m|Oui, papa.
+maman|Tes mains sont chaudes, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de gond tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1398,17 +1422,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Amir a de l'énergie. Que peut faire Victorina ?</t>
+          <t>Aniss a de l'énergie. Que fait Raphaël ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir a de l'énergie. Que peut faire Victorina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que fait Raphaël ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Loïc a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut faire Amélie ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que fait Raphaël ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1457,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut jouer. On peut attendre. Que fait Victorina ?</t>
+          <t>On peut jouer. On peut attendre. Que fait Raphaël ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1471,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,7 +1506,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,11 +1521,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1512,23 +1536,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,7 +1567,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1553,13 +1577,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_court_trop_que_fait_raphael; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Amir a de l'énergie.
-narrateur|Que peut faire Victorina ?</t>
+          <t>narrateur|Aniss a de l'énergie.
+narrateur|Que fait Raphaël ?</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina va vers maman. Maman, Amir saute. Les raisins roulent. On peut jouer. On peut attendre. On peut demander à un adulte. On pose un raisin chacun ? Oui. À tour de rôle. Maman pose un petit bol. Victorina y met des raisins. Amir s'arrête. Il souffle. Il attend son tour. Tu as demandé. Bravo, Victorina. Elle pose un raisin. Puis Amir pose un raisin. Le rond grandit. Encore un. Encore un. L'escargot apparaît. Une tête, puis la coquille. Amir attend encore. Puis il pose le dernier raisin.</t>
+          <t>Raphaël veut le ballon, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le ballon, un instant. Il écoute le gond du portail. Tu veux le ballon avec Aniss ? Papa reste à la même hauteur. Tu tiens le bord ? Aniss ne dit rien, d'abord. Il pose les mains sur le caoutchouc. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du gond. La poussière colle un peu, sous les doigts. Elle est tiède. Ils essuient le ballon sur le sol. Aniss tient le bord, plus près. Le ballon redevient plus léger, cette fois. Il roule ! Oui. Tu le vois, le ballon ? Oui, papa. Au milieu, Aniss ? J'y vais. Raphaël pousse, sans se presser. Aniss suit le ballon des yeux. Le ballon danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du portail ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina va vers maman. Maman, Amir saute. Les raisins roulent. On peut jouer. On peut attendre. On peut demander à un adulte. On pose un raisin chacun ? Oui. À tour de rôle. Maman pose un petit bol. Victorina y met des raisins. Amir s'arrête. Il souffle. Il attend son tour. Tu as demandé. Bravo, Victorina. Elle pose un raisin. Puis Amir pose un raisin. Le rond grandit. Encore un. Encore un. L'escargot apparaît. Une tête, puis la coquille. Amir attend encore. Puis il pose le dernier raisin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut le &lt;emphasis level="moderate"&gt;ballon&lt;/emphasis&gt;, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le ballon, un instant. Il écoute le gond du portail. Tu veux le ballon avec Aniss ? Papa reste à la même hauteur. Tu tiens le bord ? Aniss ne dit rien, d'abord. Il pose les mains sur le caoutchouc. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du gond. La poussière colle un peu, sous les doigts. Elle est tiède. Ils essuient le ballon sur le sol. Aniss tient le bord, plus près. Le ballon redevient plus léger, cette fois. Il roule ! Oui. Tu le vois, le ballon ? Oui, papa. Au milieu, Aniss ? J'y vais. Raphaël pousse, sans se presser. Aniss suit le ballon des yeux. Le ballon danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du portail ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Loïc a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Amélie a joué. Elle a su attendre.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël veut le &lt;emphasis&gt;ballon&lt;/emphasis&gt;, tout de suite. Je pousse, maintenant ! Il avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Attends. Aniss recule d'un pas. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le ballon, un instant. Il écoute le gond du portail. Tu veux le ballon avec Aniss ? Papa reste à la même hauteur. Tu tiens le bord ? Aniss ne dit rien, d'abord. Il pose les mains sur le caoutchouc. Je le tiens. D'accord. Merci, Raphaël. Papa a vu les deux, près du gond. La poussière colle un peu, sous les doigts. Elle est tiède. Ils essuient le ballon sur le sol. Aniss tient le bord, plus près. Le ballon redevient plus léger, cette fois. Il roule ! Oui. Tu le vois, le ballon ? Oui, papa. Au milieu, Aniss ? J'y vais. Raphaël pousse, sans se presser. Aniss suit le ballon des yeux. Le ballon danse une fois. Un. Deux. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du portail ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,18 +1667,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,30 +1701,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>ballon</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1733,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,40 +1745,64 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_ils_tiennent; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina va vers maman.
-enfant-f|Maman, Amir saute.
-enfant-f|Les raisins roulent.
-maman|On peut jouer.
-maman|On peut attendre.
-papa|On peut demander à un adulte.
-enfant-f|On pose un raisin chacun ?
-maman|Oui.
-maman|À tour de rôle.
-narrateur|Maman pose un petit bol.
-narrateur|Victorina y met des raisins.
-narrateur|Amir s'arrête.
-narrateur|Il souffle.
-narrateur|Il attend son tour.
-papa|Tu as demandé.
-papa|Bravo, Victorina.
-narrateur|Elle pose un raisin.
-narrateur|Puis Amir pose un raisin.
-narrateur|Le rond grandit.
-enfant-m|Encore un.
-enfant-f|Encore un.
-narrateur|L'escargot apparaît.
-narrateur|Une tête, puis la coquille.
-narrateur|Amir attend encore.
-narrateur|Puis il pose le dernier raisin.</t>
+          <t>narrateur|Raphaël veut le ballon, tout de suite.
+enfant-m|Je pousse, maintenant !
+narrateur|Il avance trop vite vers Aniss.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Attends.
+narrateur|Aniss recule d'un pas.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le ballon, un instant.
+narrateur|Il écoute le gond du portail.
+papa|Tu veux le ballon avec Aniss ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu tiens le bord ?
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il pose les mains sur le caoutchouc.
+copain|Je le tiens.
+enfant-m|D'accord.
+papa|Merci, Raphaël.
+narrateur|Papa a vu les deux, près du gond.
+maman|La poussière colle un peu, sous les doigts.
+enfant-m|Elle est tiède.
+narrateur|Ils essuient le ballon sur le sol.
+narrateur|Aniss tient le bord, plus près.
+narrateur|Le ballon redevient plus léger, cette fois.
+enfant-m|Il roule !
+copain|Oui.
+papa|Tu le vois, le ballon ?
+enfant-m|Oui, papa.
+maman|Au milieu, Aniss ?
+copain|J'y vais.
+narrateur|Raphaël pousse, sans se presser.
+narrateur|Aniss suit le ballon des yeux.
+narrateur|Le ballon danse une fois.
+copain|Un.
+enfant-m|Deux.
+narrateur|Le ventre de Raphaël se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du portail ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1829,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa glisse le moule au four. La porte du four fait clic. Ça sent le beurre chaud. On attend devant la vitre ? Oui. L'escargot cuit. Amir s'assoit. Ses pieds ne tapent plus. Victorina pose le bol vide. Tu as fini de poser le bol ? Oui, papa. Le nuage de farine est retombé. Le carrelage est calme. La cuillère en bois sèche. On sent le gâteau, maintenant. Il est tout chaud. Oui. L'escargot aussi.</t>
+          <t>Maman sort une caisse du coin. Elle est un peu poudreuse. Le ballon, maintenant ! Aniss court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le portail. Il est dessous ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le ballon, un instant. Il écoute le gond du portail. Sur le gond, un éclat de gond luit. Là, sur le gond. Tu tends les mains, Aniss ? Aniss ne dit rien. Il souffle, puis tend les mains. Oui. On soulève la latte ? Oui, papa. La latte sent le bois chaud. Le ballon est là, un peu tiède. Raphaël le pose près d'Aniss. Aniss le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La poussière est chaude, Aniss ? Un peu. Ils se passent le ballon, tout près. Le sol chatouille les genoux. C'est plus facile. Le portail est calme ? Oui, papa. Un rayon passe entre les lattes. Il allume le gond.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa glisse le moule au four. La porte du four fait clic. Ça sent le beurre chaud. On attend devant la vitre ? Oui. L'escargot cuit. Amir s'assoit. Ses pieds ne tapent plus. Victorina pose le bol vide. Tu as fini de poser le bol ? Oui, papa. Le nuage de farine est retombé. Le carrelage est calme. La cuillère en bois sèche. On sent le gâteau, maintenant. Il est tout chaud. Oui. L'escargot aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman sort une caisse du coin. Elle est un peu poudreuse. Le ballon, maintenant ! Aniss court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le portail. Il est dessous ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le ballon, un instant. Il écoute le gond du portail. Sur le gond, un &lt;emphasis level="moderate"&gt;éclat de gond&lt;/emphasis&gt; luit. Là, sur le gond. Tu tends les mains, Aniss ? Aniss ne dit rien. Il souffle, puis tend les mains. Oui. On soulève la latte ? Oui, papa. La latte sent le bois chaud. Le ballon est là, un peu tiède. Raphaël le pose près d'Aniss. Aniss le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La poussière est chaude, Aniss ? Un peu. Ils se passent le ballon, tout près. Le sol chatouille les genoux. C'est plus facile. Le portail est calme ? Oui, papa. Un rayon passe entre les lattes. Il allume le gond.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman prend la &lt;emphasis&gt;main&lt;/emphasis&gt; d'Amélie. Loïc range le ballon.&lt;/slow&gt; [pause]</t>
+          <t>Maman sort une caisse du coin. Elle est un peu poudreuse. Le ballon, maintenant ! Aniss court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le portail. Il est dessous ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le ballon, un instant. Il écoute le gond du portail. Sur le gond, un &lt;emphasis&gt;éclat de gond&lt;/emphasis&gt; luit. Là, sur le gond. Tu tends les mains, Aniss ? Aniss ne dit rien. Il souffle, puis tend les mains. Oui. On soulève la latte ? Oui, papa. La latte sent le bois chaud. Le ballon est là, un peu tiède. Raphaël le pose près d'Aniss. Aniss le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La poussière est chaude, Aniss ? Un peu. Ils se passent le ballon, tout près. Le sol chatouille les genoux. C'est plus facile. Le portail est calme ? Oui, papa. Un rayon passe entre les lattes. Il allume le gond. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,18 +1886,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1872,30 +1920,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de gond</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,10 +1952,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1916,29 +1964,60 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_ballon_sous_le_portail_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa glisse le moule au four.
-narrateur|La porte du four fait clic.
-narrateur|Ça sent le beurre chaud.
-maman|On attend devant la vitre ?
-enfant-f|Oui.
-enfant-f|L'escargot cuit.
-narrateur|Amir s'assoit.
-narrateur|Ses pieds ne tapent plus.
-narrateur|Victorina pose le bol vide.
-papa|Tu as fini de poser le bol ?
-enfant-f|Oui, papa.
-narrateur|Le nuage de farine est retombé.
-narrateur|Le carrelage est calme.
-narrateur|La cuillère en bois sèche.
-maman|On sent le gâteau, maintenant.
-enfant-m|Il est tout chaud.
-papa|Oui.
-papa|L'escargot aussi.</t>
+          <t>narrateur|Maman sort une caisse du coin.
+narrateur|Elle est un peu poudreuse.
+enfant-m|Le ballon, maintenant !
+narrateur|Aniss court trop, tout de suite.
+narrateur|Il saute vers le ballon.
+copain|À moi !
+narrateur|Le ballon roule sous le portail.
+enfant-m|Il est dessous !
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le ballon, un instant.
+narrateur|Il écoute le gond du portail.
+narrateur|Sur le gond, un éclat de gond luit.
+enfant-m|Là, sur le gond.
+enfant-m|Tu tends les mains, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Il souffle, puis tend les mains.
+copain|Oui.
+papa|On soulève la latte ?
+enfant-m|Oui, papa.
+narrateur|La latte sent le bois chaud.
+narrateur|Le ballon est là, un peu tiède.
+narrateur|Raphaël le pose près d'Aniss.
+narrateur|Aniss le rend, sans courir.
+enfant-m|Poumf.
+copain|Poumf.
+papa|Le ballon est bien gonflé ?
+enfant-m|Oui, papa.
+maman|La poussière est chaude, Aniss ?
+copain|Un peu.
+narrateur|Ils se passent le ballon, tout près.
+narrateur|Le sol chatouille les genoux.
+enfant-m|C'est plus facile.
+papa|Le portail est calme ?
+enfant-m|Oui, papa.
+maman|Un rayon passe entre les lattes.
+enfant-m|Il allume le gond.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2044,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot est sur le gâteau. Tout en rond. Il sent bon, maintenant. Le bol est vide.</t>
+          <t>Ils restent près du gond. Maman essuie un peu de poussière. Le ballon a roulé, papa. Tu l'as vu, toi ? Oui, près du portail. On est bien, ici. Raphaël tapote le ballon du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Raphaël. Oui, avec Aniss. Le ballon est resté. Ça sent le bois, un peu tiède. Et le gond, maman. Oui, dans l'air. Le ballon reste près du mur. Un éclat de gond tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot est sur le gâteau. Tout en rond. Il sent bon, maintenant. Le bol est vide.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du gond. Maman essuie un peu de poussière. Le ballon a roulé, papa. Tu l'as vu, toi ? Oui, près du portail. On est bien, ici. Raphaël tapote le ballon du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Raphaël. Oui, avec Aniss. Le ballon est resté. Ça sent le bois, un peu tiède. Et le gond, maman. Oui, dans l'air. Le ballon reste près du mur. Un &lt;emphasis level="moderate"&gt;éclat de gond&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du gond. Maman essuie un peu de poussière. Le ballon a roulé, papa. Tu l'as vu, toi ? Oui, près du portail. On est bien, ici. Raphaël tapote le ballon du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Raphaël. Oui, avec Aniss. Le ballon est resté. Ça sent le bois, un peu tiède. Et le gond, maman. Oui, dans l'air. Le ballon reste près du mur. Un &lt;emphasis&gt;éclat de gond&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,7 +2101,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2030,10 +2109,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2121,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,14 +2135,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de gond</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2075,11 +2158,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,27 +2171,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|L'escargot est sur le gâteau.
-maman|Tout en rond.
-papa|Il sent bon, maintenant.
-narrateur|Le bol est vide.</t>
+          <t>narrateur|Ils restent près du gond.
+narrateur|Maman essuie un peu de poussière.
+enfant-m|Le ballon a roulé, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près du portail.
+maman|On est bien, ici.
+narrateur|Raphaël tapote le ballon du doigt.
+enfant-m|Il a une trace de poussière.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le ballon est resté, Raphaël.
+enfant-m|Oui, avec Aniss.
+copain|Le ballon est resté.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-m|Et le gond, maman.
+maman|Oui, dans l'air.
+narrateur|Le ballon reste près du mur.
+narrateur|Un éclat de gond tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2186,6 +2287,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>